<commit_message>
tuning with fixed flagelates and good scrores
</commit_message>
<xml_diff>
--- a/notebooks/SHEM/tuning/eval_files/DO_model_whole_v5.xlsx
+++ b/notebooks/SHEM/tuning/eval_files/DO_model_whole_v5.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ369"/>
+  <dimension ref="A1:AR369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -631,6 +631,11 @@
           <t>pred2mine2l_z2</t>
         </is>
       </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>remin2l_z2</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -768,6 +773,9 @@
       <c r="AQ2" t="n">
         <v>262.0680847167969</v>
       </c>
+      <c r="AR2" t="n">
+        <v>256.2673034667969</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -905,6 +913,9 @@
       <c r="AQ3" t="n">
         <v>261.0550231933594</v>
       </c>
+      <c r="AR3" t="n">
+        <v>255.3670654296875</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -1044,6 +1055,9 @@
       <c r="AQ4" t="n">
         <v>256.7671203613281</v>
       </c>
+      <c r="AR4" t="n">
+        <v>252.7723693847656</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1183,6 +1197,9 @@
       <c r="AQ5" t="n">
         <v>244.8489685058594</v>
       </c>
+      <c r="AR5" t="n">
+        <v>244.1126861572266</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1320,6 +1337,9 @@
       <c r="AQ6" t="n">
         <v>234.0832061767578</v>
       </c>
+      <c r="AR6" t="n">
+        <v>233.9153594970703</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1457,6 +1477,9 @@
       <c r="AQ7" t="n">
         <v>222.9816436767578</v>
       </c>
+      <c r="AR7" t="n">
+        <v>222.0880584716797</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1594,6 +1617,9 @@
       <c r="AQ8" t="n">
         <v>208.5938110351562</v>
       </c>
+      <c r="AR8" t="n">
+        <v>208.7886657714844</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1731,6 +1757,9 @@
       <c r="AQ9" t="n">
         <v>162.700439453125</v>
       </c>
+      <c r="AR9" t="n">
+        <v>162.5455169677734</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1868,6 +1897,9 @@
       <c r="AQ10" t="n">
         <v>128.0037384033203</v>
       </c>
+      <c r="AR10" t="n">
+        <v>128.8388366699219</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -2005,6 +2037,9 @@
       <c r="AQ11" t="n">
         <v>115.9033813476562</v>
       </c>
+      <c r="AR11" t="n">
+        <v>115.5895462036133</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -2142,6 +2177,9 @@
       <c r="AQ12" t="n">
         <v>112.6076583862305</v>
       </c>
+      <c r="AR12" t="n">
+        <v>112.5818176269531</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -2277,6 +2315,9 @@
       <c r="AQ13" t="n">
         <v>111.8963851928711</v>
       </c>
+      <c r="AR13" t="n">
+        <v>111.7166976928711</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -2416,6 +2457,9 @@
       <c r="AQ14" t="n">
         <v>250.1314392089844</v>
       </c>
+      <c r="AR14" t="n">
+        <v>250.2248077392578</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2553,6 +2597,9 @@
       <c r="AQ15" t="n">
         <v>249.2201232910156</v>
       </c>
+      <c r="AR15" t="n">
+        <v>249.1802978515625</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2692,6 +2739,9 @@
       <c r="AQ16" t="n">
         <v>247.7755584716797</v>
       </c>
+      <c r="AR16" t="n">
+        <v>247.5335693359375</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2831,6 +2881,9 @@
       <c r="AQ17" t="n">
         <v>245.4962158203125</v>
       </c>
+      <c r="AR17" t="n">
+        <v>244.9562530517578</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2968,6 +3021,9 @@
       <c r="AQ18" t="n">
         <v>243.4464721679688</v>
       </c>
+      <c r="AR18" t="n">
+        <v>242.6639404296875</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -3105,6 +3161,9 @@
       <c r="AQ19" t="n">
         <v>240.7434539794922</v>
       </c>
+      <c r="AR19" t="n">
+        <v>240.2516784667969</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -3242,6 +3301,9 @@
       <c r="AQ20" t="n">
         <v>237.9414978027344</v>
       </c>
+      <c r="AR20" t="n">
+        <v>237.8082122802734</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -3379,6 +3441,9 @@
       <c r="AQ21" t="n">
         <v>233.735595703125</v>
       </c>
+      <c r="AR21" t="n">
+        <v>233.1490631103516</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -3516,6 +3581,9 @@
       <c r="AQ22" t="n">
         <v>228.8103485107422</v>
       </c>
+      <c r="AR22" t="n">
+        <v>228.8815460205078</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -3653,6 +3721,9 @@
       <c r="AQ23" t="n">
         <v>223.7301635742188</v>
       </c>
+      <c r="AR23" t="n">
+        <v>223.7552490234375</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -3790,6 +3861,9 @@
       <c r="AQ24" t="n">
         <v>249.7884368896484</v>
       </c>
+      <c r="AR24" t="n">
+        <v>250.4973297119141</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -3927,6 +4001,9 @@
       <c r="AQ25" t="n">
         <v>249.3892364501953</v>
       </c>
+      <c r="AR25" t="n">
+        <v>250.0050201416016</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -4066,6 +4143,9 @@
       <c r="AQ26" t="n">
         <v>249.0472412109375</v>
       </c>
+      <c r="AR26" t="n">
+        <v>249.5796508789062</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -4205,6 +4285,9 @@
       <c r="AQ27" t="n">
         <v>248.4543151855469</v>
       </c>
+      <c r="AR27" t="n">
+        <v>248.8810729980469</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -4342,6 +4425,9 @@
       <c r="AQ28" t="n">
         <v>247.9093780517578</v>
       </c>
+      <c r="AR28" t="n">
+        <v>248.2237548828125</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -4479,6 +4565,9 @@
       <c r="AQ29" t="n">
         <v>247.2992248535156</v>
       </c>
+      <c r="AR29" t="n">
+        <v>247.5858459472656</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -4616,6 +4705,9 @@
       <c r="AQ30" t="n">
         <v>246.7003479003906</v>
       </c>
+      <c r="AR30" t="n">
+        <v>246.9378509521484</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -4753,6 +4845,9 @@
       <c r="AQ31" t="n">
         <v>245.0892486572266</v>
       </c>
+      <c r="AR31" t="n">
+        <v>245.3047027587891</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -4890,6 +4985,9 @@
       <c r="AQ32" t="n">
         <v>243.5082855224609</v>
       </c>
+      <c r="AR32" t="n">
+        <v>243.232421875</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -5027,6 +5125,9 @@
       <c r="AQ33" t="n">
         <v>241.1322937011719</v>
       </c>
+      <c r="AR33" t="n">
+        <v>241.2108764648438</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -5164,6 +5265,9 @@
       <c r="AQ34" t="n">
         <v>239.5884857177734</v>
       </c>
+      <c r="AR34" t="n">
+        <v>239.4040374755859</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -5301,6 +5405,9 @@
       <c r="AQ35" t="n">
         <v>237.6627349853516</v>
       </c>
+      <c r="AR35" t="n">
+        <v>237.4280548095703</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -5436,6 +5543,9 @@
       <c r="AQ36" t="n">
         <v>237.3519287109375</v>
       </c>
+      <c r="AR36" t="n">
+        <v>237.1485290527344</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -5571,6 +5681,9 @@
       <c r="AQ37" t="n">
         <v>237.3519287109375</v>
       </c>
+      <c r="AR37" t="n">
+        <v>237.1485290527344</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -5710,6 +5823,9 @@
       <c r="AQ38" t="n">
         <v>285.7563781738281</v>
       </c>
+      <c r="AR38" t="n">
+        <v>284.7748107910156</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -5847,6 +5963,9 @@
       <c r="AQ39" t="n">
         <v>271.6922912597656</v>
       </c>
+      <c r="AR39" t="n">
+        <v>272.6109008789062</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -5986,6 +6105,9 @@
       <c r="AQ40" t="n">
         <v>248.9867248535156</v>
       </c>
+      <c r="AR40" t="n">
+        <v>250.9256286621094</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -6125,6 +6247,9 @@
       <c r="AQ41" t="n">
         <v>230.9423217773438</v>
       </c>
+      <c r="AR41" t="n">
+        <v>231.2053985595703</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -6262,6 +6387,9 @@
       <c r="AQ42" t="n">
         <v>218.3094940185547</v>
       </c>
+      <c r="AR42" t="n">
+        <v>217.7671203613281</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -6399,6 +6527,9 @@
       <c r="AQ43" t="n">
         <v>212.3047637939453</v>
       </c>
+      <c r="AR43" t="n">
+        <v>212.5865173339844</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -6536,6 +6667,9 @@
       <c r="AQ44" t="n">
         <v>208.3428497314453</v>
       </c>
+      <c r="AR44" t="n">
+        <v>208.644775390625</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -6673,6 +6807,9 @@
       <c r="AQ45" t="n">
         <v>201.5060577392578</v>
       </c>
+      <c r="AR45" t="n">
+        <v>201.8209381103516</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -6810,6 +6947,9 @@
       <c r="AQ46" t="n">
         <v>193.1032867431641</v>
       </c>
+      <c r="AR46" t="n">
+        <v>192.7050933837891</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -6947,6 +7087,9 @@
       <c r="AQ47" t="n">
         <v>181.3724212646484</v>
       </c>
+      <c r="AR47" t="n">
+        <v>181.6520080566406</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -7084,6 +7227,9 @@
       <c r="AQ48" t="n">
         <v>172.3790435791016</v>
       </c>
+      <c r="AR48" t="n">
+        <v>172.2066497802734</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -7221,6 +7367,9 @@
       <c r="AQ49" t="n">
         <v>158.7841491699219</v>
       </c>
+      <c r="AR49" t="n">
+        <v>158.4615478515625</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -7358,6 +7507,9 @@
       <c r="AQ50" t="n">
         <v>141.6233825683594</v>
       </c>
+      <c r="AR50" t="n">
+        <v>141.7243957519531</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -7491,6 +7643,9 @@
       <c r="AQ51" t="n">
         <v>127.0883255004883</v>
       </c>
+      <c r="AR51" t="n">
+        <v>127.0519561767578</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -7628,6 +7783,9 @@
       <c r="AQ52" t="n">
         <v>122.9352645874023</v>
       </c>
+      <c r="AR52" t="n">
+        <v>122.9405364990234</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -7763,6 +7921,9 @@
       <c r="AQ53" t="n">
         <v>122.6250762939453</v>
       </c>
+      <c r="AR53" t="n">
+        <v>122.6136245727539</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -7902,6 +8063,9 @@
       <c r="AQ54" t="n">
         <v>332.9824829101562</v>
       </c>
+      <c r="AR54" t="n">
+        <v>331.411376953125</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -8039,6 +8203,9 @@
       <c r="AQ55" t="n">
         <v>321.8724060058594</v>
       </c>
+      <c r="AR55" t="n">
+        <v>320.7661437988281</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -8178,6 +8345,9 @@
       <c r="AQ56" t="n">
         <v>303.7509460449219</v>
       </c>
+      <c r="AR56" t="n">
+        <v>302.7459716796875</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -8317,6 +8487,9 @@
       <c r="AQ57" t="n">
         <v>257.3426208496094</v>
       </c>
+      <c r="AR57" t="n">
+        <v>256.870849609375</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -8454,6 +8627,9 @@
       <c r="AQ58" t="n">
         <v>224.904052734375</v>
       </c>
+      <c r="AR58" t="n">
+        <v>225.0924224853516</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -8591,6 +8767,9 @@
       <c r="AQ59" t="n">
         <v>217.6302490234375</v>
       </c>
+      <c r="AR59" t="n">
+        <v>217.8514099121094</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -8728,6 +8907,9 @@
       <c r="AQ60" t="n">
         <v>217.6183013916016</v>
       </c>
+      <c r="AR60" t="n">
+        <v>217.8714447021484</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -8865,6 +9047,9 @@
       <c r="AQ61" t="n">
         <v>214.3911590576172</v>
       </c>
+      <c r="AR61" t="n">
+        <v>214.6491546630859</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -9002,6 +9187,9 @@
       <c r="AQ62" t="n">
         <v>194.0556640625</v>
       </c>
+      <c r="AR62" t="n">
+        <v>193.9435272216797</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -9139,6 +9327,9 @@
       <c r="AQ63" t="n">
         <v>168.4173889160156</v>
       </c>
+      <c r="AR63" t="n">
+        <v>168.4160614013672</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -9276,6 +9467,9 @@
       <c r="AQ64" t="n">
         <v>152.8575744628906</v>
       </c>
+      <c r="AR64" t="n">
+        <v>152.9312896728516</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -9413,6 +9607,9 @@
       <c r="AQ65" t="n">
         <v>138.8074493408203</v>
       </c>
+      <c r="AR65" t="n">
+        <v>138.8213195800781</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -9550,6 +9747,9 @@
       <c r="AQ66" t="n">
         <v>123.6327056884766</v>
       </c>
+      <c r="AR66" t="n">
+        <v>123.6277694702148</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -9687,6 +9887,9 @@
       <c r="AQ67" t="n">
         <v>120.4224395751953</v>
       </c>
+      <c r="AR67" t="n">
+        <v>120.4273147583008</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -9824,6 +10027,9 @@
       <c r="AQ68" t="n">
         <v>119.0530014038086</v>
       </c>
+      <c r="AR68" t="n">
+        <v>119.0562362670898</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -9959,6 +10165,9 @@
       <c r="AQ69" t="n">
         <v>117.9818725585938</v>
       </c>
+      <c r="AR69" t="n">
+        <v>117.9767532348633</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -10098,6 +10307,9 @@
       <c r="AQ70" t="n">
         <v>346.4737854003906</v>
       </c>
+      <c r="AR70" t="n">
+        <v>344.8009338378906</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -10235,6 +10447,9 @@
       <c r="AQ71" t="n">
         <v>338.6491088867188</v>
       </c>
+      <c r="AR71" t="n">
+        <v>336.9631958007812</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -10374,6 +10589,9 @@
       <c r="AQ72" t="n">
         <v>306.9670715332031</v>
       </c>
+      <c r="AR72" t="n">
+        <v>306.7290344238281</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -10513,6 +10731,9 @@
       <c r="AQ73" t="n">
         <v>241.9976806640625</v>
       </c>
+      <c r="AR73" t="n">
+        <v>242.0457611083984</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -10650,6 +10871,9 @@
       <c r="AQ74" t="n">
         <v>216.0860900878906</v>
       </c>
+      <c r="AR74" t="n">
+        <v>216.1295776367188</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -10787,6 +11011,9 @@
       <c r="AQ75" t="n">
         <v>204.2444610595703</v>
       </c>
+      <c r="AR75" t="n">
+        <v>204.3444213867188</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -10924,6 +11151,9 @@
       <c r="AQ76" t="n">
         <v>195.9544677734375</v>
       </c>
+      <c r="AR76" t="n">
+        <v>196.0630950927734</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -11061,6 +11291,9 @@
       <c r="AQ77" t="n">
         <v>189.5098571777344</v>
       </c>
+      <c r="AR77" t="n">
+        <v>189.4656829833984</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -11198,6 +11431,9 @@
       <c r="AQ78" t="n">
         <v>181.9656219482422</v>
       </c>
+      <c r="AR78" t="n">
+        <v>181.9684295654297</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -11335,6 +11571,9 @@
       <c r="AQ79" t="n">
         <v>166.1799621582031</v>
       </c>
+      <c r="AR79" t="n">
+        <v>166.1927490234375</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -11472,6 +11711,9 @@
       <c r="AQ80" t="n">
         <v>151.2950744628906</v>
       </c>
+      <c r="AR80" t="n">
+        <v>151.3187408447266</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -11609,6 +11851,9 @@
       <c r="AQ81" t="n">
         <v>139.3582763671875</v>
       </c>
+      <c r="AR81" t="n">
+        <v>139.3772277832031</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -11746,6 +11991,9 @@
       <c r="AQ82" t="n">
         <v>131.0723114013672</v>
       </c>
+      <c r="AR82" t="n">
+        <v>131.0823516845703</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -11883,6 +12131,9 @@
       <c r="AQ83" t="n">
         <v>124.2402038574219</v>
       </c>
+      <c r="AR83" t="n">
+        <v>124.2545623779297</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -12022,6 +12273,9 @@
       <c r="AQ84" t="n">
         <v>257.7669067382812</v>
       </c>
+      <c r="AR84" t="n">
+        <v>257.2530822753906</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -12159,6 +12413,9 @@
       <c r="AQ85" t="n">
         <v>256.5248718261719</v>
       </c>
+      <c r="AR85" t="n">
+        <v>256.1235961914062</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -12298,6 +12555,9 @@
       <c r="AQ86" t="n">
         <v>254.7588043212891</v>
       </c>
+      <c r="AR86" t="n">
+        <v>254.0724487304688</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -12437,6 +12697,9 @@
       <c r="AQ87" t="n">
         <v>252.2383728027344</v>
       </c>
+      <c r="AR87" t="n">
+        <v>251.654296875</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -12574,6 +12837,9 @@
       <c r="AQ88" t="n">
         <v>250.1525268554688</v>
       </c>
+      <c r="AR88" t="n">
+        <v>249.6475982666016</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -12711,6 +12977,9 @@
       <c r="AQ89" t="n">
         <v>247.2802734375</v>
       </c>
+      <c r="AR89" t="n">
+        <v>247.2785949707031</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -12848,6 +13117,9 @@
       <c r="AQ90" t="n">
         <v>244.8188629150391</v>
       </c>
+      <c r="AR90" t="n">
+        <v>244.8858795166016</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -12985,6 +13257,9 @@
       <c r="AQ91" t="n">
         <v>239.5846099853516</v>
       </c>
+      <c r="AR91" t="n">
+        <v>239.3096618652344</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -13122,6 +13397,9 @@
       <c r="AQ92" t="n">
         <v>235.1463165283203</v>
       </c>
+      <c r="AR92" t="n">
+        <v>235.3067474365234</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -13259,6 +13537,9 @@
       <c r="AQ93" t="n">
         <v>230.7371520996094</v>
       </c>
+      <c r="AR93" t="n">
+        <v>231.0144958496094</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -13396,6 +13677,9 @@
       <c r="AQ94" t="n">
         <v>226.2620391845703</v>
       </c>
+      <c r="AR94" t="n">
+        <v>226.7765808105469</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -13533,6 +13817,9 @@
       <c r="AQ95" t="n">
         <v>222.9390258789062</v>
       </c>
+      <c r="AR95" t="n">
+        <v>222.0737762451172</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -13670,6 +13957,9 @@
       <c r="AQ96" t="n">
         <v>218.7301940917969</v>
       </c>
+      <c r="AR96" t="n">
+        <v>218.0177001953125</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -13809,6 +14099,9 @@
       <c r="AQ97" t="n">
         <v>244.7594451904297</v>
       </c>
+      <c r="AR97" t="n">
+        <v>244.2238006591797</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -13946,6 +14239,9 @@
       <c r="AQ98" t="n">
         <v>242.0281982421875</v>
       </c>
+      <c r="AR98" t="n">
+        <v>242.2521057128906</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -14085,6 +14381,9 @@
       <c r="AQ99" t="n">
         <v>237.9898376464844</v>
       </c>
+      <c r="AR99" t="n">
+        <v>238.492919921875</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -14224,6 +14523,9 @@
       <c r="AQ100" t="n">
         <v>228.583251953125</v>
       </c>
+      <c r="AR100" t="n">
+        <v>228.7138519287109</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -14361,6 +14663,9 @@
       <c r="AQ101" t="n">
         <v>220.0376281738281</v>
       </c>
+      <c r="AR101" t="n">
+        <v>219.3501129150391</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -14498,6 +14803,9 @@
       <c r="AQ102" t="n">
         <v>212.9238128662109</v>
       </c>
+      <c r="AR102" t="n">
+        <v>212.9607696533203</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -14635,6 +14943,9 @@
       <c r="AQ103" t="n">
         <v>204.5393371582031</v>
       </c>
+      <c r="AR103" t="n">
+        <v>204.6163482666016</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -14772,6 +15083,9 @@
       <c r="AQ104" t="n">
         <v>162.1560821533203</v>
       </c>
+      <c r="AR104" t="n">
+        <v>163.8090515136719</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -14909,6 +15223,9 @@
       <c r="AQ105" t="n">
         <v>121.0380706787109</v>
       </c>
+      <c r="AR105" t="n">
+        <v>123.0475463867188</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -15046,6 +15363,9 @@
       <c r="AQ106" t="n">
         <v>107.5980606079102</v>
       </c>
+      <c r="AR106" t="n">
+        <v>107.2066116333008</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -15183,6 +15503,9 @@
       <c r="AQ107" t="n">
         <v>103.5924224853516</v>
       </c>
+      <c r="AR107" t="n">
+        <v>103.641975402832</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -15318,6 +15641,9 @@
       <c r="AQ108" t="n">
         <v>102.3597793579102</v>
       </c>
+      <c r="AR108" t="n">
+        <v>102.5878829956055</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -15455,6 +15781,9 @@
       <c r="AQ109" t="n">
         <v>253.0090942382812</v>
       </c>
+      <c r="AR109" t="n">
+        <v>265.755126953125</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -15594,6 +15923,9 @@
       <c r="AQ110" t="n">
         <v>249.1083526611328</v>
       </c>
+      <c r="AR110" t="n">
+        <v>262.0691528320312</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -15733,6 +16065,9 @@
       <c r="AQ111" t="n">
         <v>242.2103576660156</v>
       </c>
+      <c r="AR111" t="n">
+        <v>253.2514495849609</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -15870,6 +16205,9 @@
       <c r="AQ112" t="n">
         <v>230.1439208984375</v>
       </c>
+      <c r="AR112" t="n">
+        <v>232.2744445800781</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -16007,6 +16345,9 @@
       <c r="AQ113" t="n">
         <v>223.6331634521484</v>
       </c>
+      <c r="AR113" t="n">
+        <v>224.0731506347656</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -16144,6 +16485,9 @@
       <c r="AQ114" t="n">
         <v>217.0789337158203</v>
       </c>
+      <c r="AR114" t="n">
+        <v>217.2920532226562</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -16281,6 +16625,9 @@
       <c r="AQ115" t="n">
         <v>207.9734954833984</v>
       </c>
+      <c r="AR115" t="n">
+        <v>205.8597412109375</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -16418,6 +16765,9 @@
       <c r="AQ116" t="n">
         <v>169.1677093505859</v>
       </c>
+      <c r="AR116" t="n">
+        <v>165.0250701904297</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -16555,6 +16905,9 @@
       <c r="AQ117" t="n">
         <v>127.257698059082</v>
       </c>
+      <c r="AR117" t="n">
+        <v>125.3357543945312</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -16692,6 +17045,9 @@
       <c r="AQ118" t="n">
         <v>97.1551513671875</v>
       </c>
+      <c r="AR118" t="n">
+        <v>97.13176727294922</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -16829,6 +17185,9 @@
       <c r="AQ119" t="n">
         <v>89.58565521240234</v>
       </c>
+      <c r="AR119" t="n">
+        <v>90.03854370117188</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -16964,6 +17323,9 @@
       <c r="AQ120" t="n">
         <v>88.20697784423828</v>
       </c>
+      <c r="AR120" t="n">
+        <v>88.55929565429688</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -17099,6 +17461,9 @@
       <c r="AQ121" t="n">
         <v>88.20697784423828</v>
       </c>
+      <c r="AR121" t="n">
+        <v>88.55929565429688</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -17238,6 +17603,9 @@
       <c r="AQ122" t="n">
         <v>251.1114349365234</v>
       </c>
+      <c r="AR122" t="n">
+        <v>250.6402130126953</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -17375,6 +17743,9 @@
       <c r="AQ123" t="n">
         <v>248.7686462402344</v>
       </c>
+      <c r="AR123" t="n">
+        <v>248.5930786132812</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -17514,6 +17885,9 @@
       <c r="AQ124" t="n">
         <v>244.7375640869141</v>
       </c>
+      <c r="AR124" t="n">
+        <v>245.3470458984375</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -17653,6 +18027,9 @@
       <c r="AQ125" t="n">
         <v>237.9969482421875</v>
       </c>
+      <c r="AR125" t="n">
+        <v>237.91552734375</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -17790,6 +18167,9 @@
       <c r="AQ126" t="n">
         <v>230.8541870117188</v>
       </c>
+      <c r="AR126" t="n">
+        <v>230.1894378662109</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -17927,6 +18307,9 @@
       <c r="AQ127" t="n">
         <v>199.5291442871094</v>
       </c>
+      <c r="AR127" t="n">
+        <v>198.0053863525391</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -18064,6 +18447,9 @@
       <c r="AQ128" t="n">
         <v>161.5022735595703</v>
       </c>
+      <c r="AR128" t="n">
+        <v>160.2871551513672</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -18201,6 +18587,9 @@
       <c r="AQ129" t="n">
         <v>142.5924377441406</v>
       </c>
+      <c r="AR129" t="n">
+        <v>143.2570037841797</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -18340,6 +18729,9 @@
       <c r="AQ130" t="n">
         <v>260.0207824707031</v>
       </c>
+      <c r="AR130" t="n">
+        <v>259.7715148925781</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -18477,6 +18869,9 @@
       <c r="AQ131" t="n">
         <v>259.5014343261719</v>
       </c>
+      <c r="AR131" t="n">
+        <v>259.2063598632812</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -18616,6 +19011,9 @@
       <c r="AQ132" t="n">
         <v>257.9131164550781</v>
       </c>
+      <c r="AR132" t="n">
+        <v>257.371826171875</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -18755,6 +19153,9 @@
       <c r="AQ133" t="n">
         <v>251.0269470214844</v>
       </c>
+      <c r="AR133" t="n">
+        <v>250.4154357910156</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -18892,6 +19293,9 @@
       <c r="AQ134" t="n">
         <v>240.108642578125</v>
       </c>
+      <c r="AR134" t="n">
+        <v>239.0070495605469</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -19029,6 +19433,9 @@
       <c r="AQ135" t="n">
         <v>228.1832122802734</v>
       </c>
+      <c r="AR135" t="n">
+        <v>227.3891448974609</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -19166,6 +19573,9 @@
       <c r="AQ136" t="n">
         <v>217.7462005615234</v>
       </c>
+      <c r="AR136" t="n">
+        <v>216.8210144042969</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -19303,6 +19713,9 @@
       <c r="AQ137" t="n">
         <v>181.0137939453125</v>
       </c>
+      <c r="AR137" t="n">
+        <v>181.1633911132812</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -19440,6 +19853,9 @@
       <c r="AQ138" t="n">
         <v>158.4276428222656</v>
       </c>
+      <c r="AR138" t="n">
+        <v>158.1509246826172</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -19577,6 +19993,9 @@
       <c r="AQ139" t="n">
         <v>153.1020965576172</v>
       </c>
+      <c r="AR139" t="n">
+        <v>152.8914337158203</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -19716,6 +20135,9 @@
       <c r="AQ140" t="n">
         <v>255.0591888427734</v>
       </c>
+      <c r="AR140" t="n">
+        <v>254.5875854492188</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -19853,6 +20275,9 @@
       <c r="AQ141" t="n">
         <v>254.1183471679688</v>
       </c>
+      <c r="AR141" t="n">
+        <v>253.6757049560547</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -19992,6 +20417,9 @@
       <c r="AQ142" t="n">
         <v>252.7680206298828</v>
       </c>
+      <c r="AR142" t="n">
+        <v>251.7468719482422</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -20131,6 +20559,9 @@
       <c r="AQ143" t="n">
         <v>249.6813201904297</v>
       </c>
+      <c r="AR143" t="n">
+        <v>248.4284362792969</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -20268,6 +20699,9 @@
       <c r="AQ144" t="n">
         <v>247.6762542724609</v>
       </c>
+      <c r="AR144" t="n">
+        <v>246.3040313720703</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -20405,6 +20839,9 @@
       <c r="AQ145" t="n">
         <v>245.6646270751953</v>
       </c>
+      <c r="AR145" t="n">
+        <v>244.4445190429688</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -20542,6 +20979,9 @@
       <c r="AQ146" t="n">
         <v>243.8004913330078</v>
       </c>
+      <c r="AR146" t="n">
+        <v>242.8882598876953</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -20679,6 +21119,9 @@
       <c r="AQ147" t="n">
         <v>240.5704803466797</v>
       </c>
+      <c r="AR147" t="n">
+        <v>239.9824829101562</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -20816,6 +21259,9 @@
       <c r="AQ148" t="n">
         <v>236.2742767333984</v>
       </c>
+      <c r="AR148" t="n">
+        <v>235.4811706542969</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -20953,6 +21399,9 @@
       <c r="AQ149" t="n">
         <v>233.2590026855469</v>
       </c>
+      <c r="AR149" t="n">
+        <v>232.6151123046875</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -21090,6 +21539,9 @@
       <c r="AQ150" t="n">
         <v>228.35595703125</v>
       </c>
+      <c r="AR150" t="n">
+        <v>228.2901763916016</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -21225,6 +21677,9 @@
       <c r="AQ151" t="n">
         <v>227.8688354492188</v>
       </c>
+      <c r="AR151" t="n">
+        <v>227.8285980224609</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -21364,6 +21819,9 @@
       <c r="AQ152" t="n">
         <v>271.3934631347656</v>
       </c>
+      <c r="AR152" t="n">
+        <v>270.1452941894531</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -21501,6 +21959,9 @@
       <c r="AQ153" t="n">
         <v>269.7562866210938</v>
       </c>
+      <c r="AR153" t="n">
+        <v>269.7671508789062</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -21640,6 +22101,9 @@
       <c r="AQ154" t="n">
         <v>262.3706359863281</v>
       </c>
+      <c r="AR154" t="n">
+        <v>263.9187316894531</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -21779,6 +22243,9 @@
       <c r="AQ155" t="n">
         <v>251.9368133544922</v>
       </c>
+      <c r="AR155" t="n">
+        <v>249.1669769287109</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -21916,6 +22383,9 @@
       <c r="AQ156" t="n">
         <v>246.2222900390625</v>
       </c>
+      <c r="AR156" t="n">
+        <v>243.831787109375</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -22053,6 +22523,9 @@
       <c r="AQ157" t="n">
         <v>241.3152465820312</v>
       </c>
+      <c r="AR157" t="n">
+        <v>240.6497802734375</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -22190,6 +22663,9 @@
       <c r="AQ158" t="n">
         <v>238.2080535888672</v>
       </c>
+      <c r="AR158" t="n">
+        <v>238.2980041503906</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -22327,6 +22803,9 @@
       <c r="AQ159" t="n">
         <v>232.2137908935547</v>
       </c>
+      <c r="AR159" t="n">
+        <v>232.1455841064453</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -22464,6 +22943,9 @@
       <c r="AQ160" t="n">
         <v>224.4955291748047</v>
       </c>
+      <c r="AR160" t="n">
+        <v>222.5382537841797</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -22601,6 +23083,9 @@
       <c r="AQ161" t="n">
         <v>211.6408081054688</v>
       </c>
+      <c r="AR161" t="n">
+        <v>208.5818786621094</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -22738,6 +23223,9 @@
       <c r="AQ162" t="n">
         <v>194.1608734130859</v>
       </c>
+      <c r="AR162" t="n">
+        <v>188.0726470947266</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -22873,6 +23361,9 @@
       <c r="AQ163" t="n">
         <v>186.8420562744141</v>
       </c>
+      <c r="AR163" t="n">
+        <v>181.8278503417969</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -23012,6 +23503,9 @@
       <c r="AQ164" t="n">
         <v>306.7363586425781</v>
       </c>
+      <c r="AR164" t="n">
+        <v>305.5714416503906</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -23149,6 +23643,9 @@
       <c r="AQ165" t="n">
         <v>305.6953735351562</v>
       </c>
+      <c r="AR165" t="n">
+        <v>305.3453063964844</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -23288,6 +23785,9 @@
       <c r="AQ166" t="n">
         <v>293.3990173339844</v>
       </c>
+      <c r="AR166" t="n">
+        <v>271.5547180175781</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -23427,6 +23927,9 @@
       <c r="AQ167" t="n">
         <v>232.5676116943359</v>
       </c>
+      <c r="AR167" t="n">
+        <v>229.2540283203125</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -23564,6 +24067,9 @@
       <c r="AQ168" t="n">
         <v>219.8595428466797</v>
       </c>
+      <c r="AR168" t="n">
+        <v>211.0418548583984</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -23701,6 +24207,9 @@
       <c r="AQ169" t="n">
         <v>218.0081634521484</v>
       </c>
+      <c r="AR169" t="n">
+        <v>209.2685852050781</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -23838,6 +24347,9 @@
       <c r="AQ170" t="n">
         <v>221.8043365478516</v>
       </c>
+      <c r="AR170" t="n">
+        <v>211.0040435791016</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -23975,6 +24487,9 @@
       <c r="AQ171" t="n">
         <v>228.0464477539062</v>
       </c>
+      <c r="AR171" t="n">
+        <v>219.8551788330078</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -24112,6 +24627,9 @@
       <c r="AQ172" t="n">
         <v>217.2117919921875</v>
       </c>
+      <c r="AR172" t="n">
+        <v>215.6331329345703</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -24249,6 +24767,9 @@
       <c r="AQ173" t="n">
         <v>203.6577301025391</v>
       </c>
+      <c r="AR173" t="n">
+        <v>204.8713073730469</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -24386,6 +24907,9 @@
       <c r="AQ174" t="n">
         <v>188.2076568603516</v>
       </c>
+      <c r="AR174" t="n">
+        <v>191.4385528564453</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -24523,6 +25047,9 @@
       <c r="AQ175" t="n">
         <v>154.6918029785156</v>
       </c>
+      <c r="AR175" t="n">
+        <v>149.6206970214844</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -24660,6 +25187,9 @@
       <c r="AQ176" t="n">
         <v>135.5968475341797</v>
       </c>
+      <c r="AR176" t="n">
+        <v>131.9368438720703</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -24797,6 +25327,9 @@
       <c r="AQ177" t="n">
         <v>126.2803039550781</v>
       </c>
+      <c r="AR177" t="n">
+        <v>123.3895721435547</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -24932,6 +25465,9 @@
       <c r="AQ178" t="n">
         <v>125.2969589233398</v>
       </c>
+      <c r="AR178" t="n">
+        <v>122.5783920288086</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -25071,6 +25607,9 @@
       <c r="AQ179" t="n">
         <v>272.7333374023438</v>
       </c>
+      <c r="AR179" t="n">
+        <v>266.8895568847656</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -25208,6 +25747,9 @@
       <c r="AQ180" t="n">
         <v>261.7883605957031</v>
       </c>
+      <c r="AR180" t="n">
+        <v>259.3447875976562</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -25347,6 +25889,9 @@
       <c r="AQ181" t="n">
         <v>254.9080505371094</v>
       </c>
+      <c r="AR181" t="n">
+        <v>252.2922058105469</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -25486,6 +26031,9 @@
       <c r="AQ182" t="n">
         <v>231.5428314208984</v>
       </c>
+      <c r="AR182" t="n">
+        <v>242.9333648681641</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -25623,6 +26171,9 @@
       <c r="AQ183" t="n">
         <v>210.5791778564453</v>
       </c>
+      <c r="AR183" t="n">
+        <v>213.8651733398438</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -25760,6 +26311,9 @@
       <c r="AQ184" t="n">
         <v>202.8966217041016</v>
       </c>
+      <c r="AR184" t="n">
+        <v>202.0540771484375</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -25897,6 +26451,9 @@
       <c r="AQ185" t="n">
         <v>200.6593780517578</v>
       </c>
+      <c r="AR185" t="n">
+        <v>200.9973907470703</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -26034,6 +26591,9 @@
       <c r="AQ186" t="n">
         <v>195.8523559570312</v>
       </c>
+      <c r="AR186" t="n">
+        <v>198.4087677001953</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -26171,6 +26731,9 @@
       <c r="AQ187" t="n">
         <v>187.314453125</v>
       </c>
+      <c r="AR187" t="n">
+        <v>189.2635803222656</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -26308,6 +26871,9 @@
       <c r="AQ188" t="n">
         <v>180.5932464599609</v>
       </c>
+      <c r="AR188" t="n">
+        <v>182.3375091552734</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -26445,6 +27011,9 @@
       <c r="AQ189" t="n">
         <v>175.9275207519531</v>
       </c>
+      <c r="AR189" t="n">
+        <v>175.4894714355469</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -26582,6 +27151,9 @@
       <c r="AQ190" t="n">
         <v>148.942138671875</v>
       </c>
+      <c r="AR190" t="n">
+        <v>156.6001281738281</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -26719,6 +27291,9 @@
       <c r="AQ191" t="n">
         <v>127.0700225830078</v>
       </c>
+      <c r="AR191" t="n">
+        <v>126.9455795288086</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -26856,6 +27431,9 @@
       <c r="AQ192" t="n">
         <v>118.0815124511719</v>
       </c>
+      <c r="AR192" t="n">
+        <v>117.2281188964844</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -26991,6 +27569,9 @@
       <c r="AQ193" t="n">
         <v>117.6649856567383</v>
       </c>
+      <c r="AR193" t="n">
+        <v>116.8481903076172</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -27130,6 +27711,9 @@
       <c r="AQ194" t="n">
         <v>309.9607238769531</v>
       </c>
+      <c r="AR194" t="n">
+        <v>323.9445190429688</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -27267,6 +27851,9 @@
       <c r="AQ195" t="n">
         <v>303.5990295410156</v>
       </c>
+      <c r="AR195" t="n">
+        <v>323.8247985839844</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -27406,6 +27993,9 @@
       <c r="AQ196" t="n">
         <v>284.9744262695312</v>
       </c>
+      <c r="AR196" t="n">
+        <v>317.3212280273438</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -27545,6 +28135,9 @@
       <c r="AQ197" t="n">
         <v>222.2541198730469</v>
       </c>
+      <c r="AR197" t="n">
+        <v>250.9610595703125</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -27682,6 +28275,9 @@
       <c r="AQ198" t="n">
         <v>200.5995025634766</v>
       </c>
+      <c r="AR198" t="n">
+        <v>222.4837951660156</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -27819,6 +28415,9 @@
       <c r="AQ199" t="n">
         <v>195.7839508056641</v>
       </c>
+      <c r="AR199" t="n">
+        <v>204.3610534667969</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -27956,6 +28555,9 @@
       <c r="AQ200" t="n">
         <v>195.9093170166016</v>
       </c>
+      <c r="AR200" t="n">
+        <v>196.4994812011719</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -28093,6 +28695,9 @@
       <c r="AQ201" t="n">
         <v>199.1134033203125</v>
       </c>
+      <c r="AR201" t="n">
+        <v>196.5790252685547</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -28230,6 +28835,9 @@
       <c r="AQ202" t="n">
         <v>200.3454895019531</v>
       </c>
+      <c r="AR202" t="n">
+        <v>196.4978790283203</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -28367,6 +28975,9 @@
       <c r="AQ203" t="n">
         <v>195.8822784423828</v>
       </c>
+      <c r="AR203" t="n">
+        <v>190.7017211914062</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -28504,6 +29115,9 @@
       <c r="AQ204" t="n">
         <v>186.4566802978516</v>
       </c>
+      <c r="AR204" t="n">
+        <v>178.1794128417969</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -28641,6 +29255,9 @@
       <c r="AQ205" t="n">
         <v>167.2699584960938</v>
       </c>
+      <c r="AR205" t="n">
+        <v>156.9233856201172</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -28778,6 +29395,9 @@
       <c r="AQ206" t="n">
         <v>142.0613861083984</v>
       </c>
+      <c r="AR206" t="n">
+        <v>137.3950958251953</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -28915,6 +29535,9 @@
       <c r="AQ207" t="n">
         <v>124.0054016113281</v>
       </c>
+      <c r="AR207" t="n">
+        <v>124.0522613525391</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -29052,6 +29675,9 @@
       <c r="AQ208" t="n">
         <v>120.6952056884766</v>
       </c>
+      <c r="AR208" t="n">
+        <v>120.8503341674805</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -29189,6 +29815,9 @@
       <c r="AQ209" t="n">
         <v>117.6396026611328</v>
       </c>
+      <c r="AR209" t="n">
+        <v>117.4237747192383</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -29328,6 +29957,9 @@
       <c r="AQ210" t="n">
         <v>292.8783874511719</v>
       </c>
+      <c r="AR210" t="n">
+        <v>306.2963256835938</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -29465,6 +30097,9 @@
       <c r="AQ211" t="n">
         <v>283.3854675292969</v>
       </c>
+      <c r="AR211" t="n">
+        <v>283.2688293457031</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -29604,6 +30239,9 @@
       <c r="AQ212" t="n">
         <v>271.4242858886719</v>
       </c>
+      <c r="AR212" t="n">
+        <v>254.5145874023438</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -29743,6 +30381,9 @@
       <c r="AQ213" t="n">
         <v>242.902587890625</v>
       </c>
+      <c r="AR213" t="n">
+        <v>241.0866851806641</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -29880,6 +30521,9 @@
       <c r="AQ214" t="n">
         <v>215.7812347412109</v>
       </c>
+      <c r="AR214" t="n">
+        <v>224.8701019287109</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -30017,6 +30661,9 @@
       <c r="AQ215" t="n">
         <v>192.6676635742188</v>
       </c>
+      <c r="AR215" t="n">
+        <v>197.8583221435547</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -30154,6 +30801,9 @@
       <c r="AQ216" t="n">
         <v>183.7925720214844</v>
       </c>
+      <c r="AR216" t="n">
+        <v>185.3584136962891</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -30291,6 +30941,9 @@
       <c r="AQ217" t="n">
         <v>186.2534332275391</v>
       </c>
+      <c r="AR217" t="n">
+        <v>184.2375793457031</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -30428,6 +31081,9 @@
       <c r="AQ218" t="n">
         <v>189.7674102783203</v>
       </c>
+      <c r="AR218" t="n">
+        <v>188.8643646240234</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -30561,6 +31217,9 @@
       <c r="AQ219" t="n">
         <v>184.4860687255859</v>
       </c>
+      <c r="AR219" t="n">
+        <v>185.2541046142578</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -30698,6 +31357,9 @@
       <c r="AQ220" t="n">
         <v>171.8751068115234</v>
       </c>
+      <c r="AR220" t="n">
+        <v>169.089111328125</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -30835,6 +31497,9 @@
       <c r="AQ221" t="n">
         <v>161.3912353515625</v>
       </c>
+      <c r="AR221" t="n">
+        <v>156.5706939697266</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -30972,6 +31637,9 @@
       <c r="AQ222" t="n">
         <v>143.2927703857422</v>
       </c>
+      <c r="AR222" t="n">
+        <v>143.1573638916016</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -31109,6 +31777,9 @@
       <c r="AQ223" t="n">
         <v>124.1707000732422</v>
       </c>
+      <c r="AR223" t="n">
+        <v>124.8965072631836</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -31246,6 +31917,9 @@
       <c r="AQ224" t="n">
         <v>120.1332397460938</v>
       </c>
+      <c r="AR224" t="n">
+        <v>120.5600204467773</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -31385,6 +32059,9 @@
       <c r="AQ225" t="n">
         <v>232.3046722412109</v>
       </c>
+      <c r="AR225" t="n">
+        <v>237.8023986816406</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -31524,6 +32201,9 @@
       <c r="AQ226" t="n">
         <v>223.5668792724609</v>
       </c>
+      <c r="AR226" t="n">
+        <v>232.1842956542969</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -31661,6 +32341,9 @@
       <c r="AQ227" t="n">
         <v>217.0124664306641</v>
       </c>
+      <c r="AR227" t="n">
+        <v>219.635009765625</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -31798,6 +32481,9 @@
       <c r="AQ228" t="n">
         <v>211.9018707275391</v>
       </c>
+      <c r="AR228" t="n">
+        <v>211.3098907470703</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -31935,6 +32621,9 @@
       <c r="AQ229" t="n">
         <v>206.1741790771484</v>
       </c>
+      <c r="AR229" t="n">
+        <v>205.2371520996094</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -32072,6 +32761,9 @@
       <c r="AQ230" t="n">
         <v>200.4791870117188</v>
       </c>
+      <c r="AR230" t="n">
+        <v>199.1480712890625</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -32209,6 +32901,9 @@
       <c r="AQ231" t="n">
         <v>183.2615509033203</v>
       </c>
+      <c r="AR231" t="n">
+        <v>183.9553070068359</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -32346,6 +33041,9 @@
       <c r="AQ232" t="n">
         <v>172.6601715087891</v>
       </c>
+      <c r="AR232" t="n">
+        <v>173.5259399414062</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -32483,6 +33181,9 @@
       <c r="AQ233" t="n">
         <v>157.8214111328125</v>
       </c>
+      <c r="AR233" t="n">
+        <v>157.5553436279297</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -32618,6 +33319,9 @@
       <c r="AQ234" t="n">
         <v>151.4927673339844</v>
       </c>
+      <c r="AR234" t="n">
+        <v>150.9799041748047</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -32757,6 +33461,9 @@
       <c r="AQ235" t="n">
         <v>242.1210784912109</v>
       </c>
+      <c r="AR235" t="n">
+        <v>260.9752197265625</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -32894,6 +33601,9 @@
       <c r="AQ236" t="n">
         <v>240.8523559570312</v>
       </c>
+      <c r="AR236" t="n">
+        <v>255.9464263916016</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -33033,6 +33743,9 @@
       <c r="AQ237" t="n">
         <v>238.6600646972656</v>
       </c>
+      <c r="AR237" t="n">
+        <v>246.0466613769531</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -33172,6 +33885,9 @@
       <c r="AQ238" t="n">
         <v>227.0796813964844</v>
       </c>
+      <c r="AR238" t="n">
+        <v>228.5512084960938</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -33309,6 +34025,9 @@
       <c r="AQ239" t="n">
         <v>213.8596649169922</v>
       </c>
+      <c r="AR239" t="n">
+        <v>213.6457061767578</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -33446,6 +34165,9 @@
       <c r="AQ240" t="n">
         <v>199.5381317138672</v>
       </c>
+      <c r="AR240" t="n">
+        <v>203.7781829833984</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -33583,6 +34305,9 @@
       <c r="AQ241" t="n">
         <v>184.8677673339844</v>
       </c>
+      <c r="AR241" t="n">
+        <v>185.7754516601562</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -33720,6 +34445,9 @@
       <c r="AQ242" t="n">
         <v>163.7164764404297</v>
       </c>
+      <c r="AR242" t="n">
+        <v>163.4333343505859</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -33857,6 +34585,9 @@
       <c r="AQ243" t="n">
         <v>156.2080383300781</v>
       </c>
+      <c r="AR243" t="n">
+        <v>154.6628265380859</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -33994,6 +34725,9 @@
       <c r="AQ244" t="n">
         <v>149.4994506835938</v>
       </c>
+      <c r="AR244" t="n">
+        <v>149.0706176757812</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -34131,6 +34865,9 @@
       <c r="AQ245" t="n">
         <v>144.8677978515625</v>
       </c>
+      <c r="AR245" t="n">
+        <v>144.9373474121094</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -34268,6 +35005,9 @@
       <c r="AQ246" t="n">
         <v>142.6173400878906</v>
       </c>
+      <c r="AR246" t="n">
+        <v>142.7336120605469</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -34405,6 +35145,9 @@
       <c r="AQ247" t="n">
         <v>137.9266357421875</v>
       </c>
+      <c r="AR247" t="n">
+        <v>138.3127593994141</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -34540,6 +35283,9 @@
       <c r="AQ248" t="n">
         <v>133.7201538085938</v>
       </c>
+      <c r="AR248" t="n">
+        <v>134.2080688476562</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -34679,6 +35425,9 @@
       <c r="AQ249" t="n">
         <v>289.2169799804688</v>
       </c>
+      <c r="AR249" t="n">
+        <v>292.8893432617188</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -34816,6 +35565,9 @@
       <c r="AQ250" t="n">
         <v>286.265380859375</v>
       </c>
+      <c r="AR250" t="n">
+        <v>289.2093200683594</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -34955,6 +35707,9 @@
       <c r="AQ251" t="n">
         <v>279.5610961914062</v>
       </c>
+      <c r="AR251" t="n">
+        <v>283.1177368164062</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -35094,6 +35849,9 @@
       <c r="AQ252" t="n">
         <v>269.9946899414062</v>
       </c>
+      <c r="AR252" t="n">
+        <v>278.3284301757812</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -35231,6 +35989,9 @@
       <c r="AQ253" t="n">
         <v>249.2847290039062</v>
       </c>
+      <c r="AR253" t="n">
+        <v>256.5410766601562</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -35368,6 +36129,9 @@
       <c r="AQ254" t="n">
         <v>212.62890625</v>
       </c>
+      <c r="AR254" t="n">
+        <v>214.3679046630859</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -35505,6 +36269,9 @@
       <c r="AQ255" t="n">
         <v>191.6920776367188</v>
       </c>
+      <c r="AR255" t="n">
+        <v>187.3507232666016</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -35642,6 +36409,9 @@
       <c r="AQ256" t="n">
         <v>170.2998962402344</v>
       </c>
+      <c r="AR256" t="n">
+        <v>169.3006896972656</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -35779,6 +36549,9 @@
       <c r="AQ257" t="n">
         <v>162.6673736572266</v>
       </c>
+      <c r="AR257" t="n">
+        <v>164.2920227050781</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -35916,6 +36689,9 @@
       <c r="AQ258" t="n">
         <v>156.9312591552734</v>
       </c>
+      <c r="AR258" t="n">
+        <v>157.3339538574219</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -36053,6 +36829,9 @@
       <c r="AQ259" t="n">
         <v>149.0867614746094</v>
       </c>
+      <c r="AR259" t="n">
+        <v>148.5977783203125</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -36190,6 +36969,9 @@
       <c r="AQ260" t="n">
         <v>144.4866333007812</v>
       </c>
+      <c r="AR260" t="n">
+        <v>145.0011291503906</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -36327,6 +37109,9 @@
       <c r="AQ261" t="n">
         <v>144.9418334960938</v>
       </c>
+      <c r="AR261" t="n">
+        <v>144.9821014404297</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -36464,6 +37249,9 @@
       <c r="AQ262" t="n">
         <v>139.3552856445312</v>
       </c>
+      <c r="AR262" t="n">
+        <v>139.0249481201172</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -36601,6 +37389,9 @@
       <c r="AQ263" t="n">
         <v>129.0667724609375</v>
       </c>
+      <c r="AR263" t="n">
+        <v>128.4129180908203</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -36738,6 +37529,9 @@
       <c r="AQ264" t="n">
         <v>115.1986083984375</v>
       </c>
+      <c r="AR264" t="n">
+        <v>114.722053527832</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -36877,6 +37671,9 @@
       <c r="AQ265" t="n">
         <v>265.0675659179688</v>
       </c>
+      <c r="AR265" t="n">
+        <v>269.5375671386719</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -37014,6 +37811,9 @@
       <c r="AQ266" t="n">
         <v>263.6190185546875</v>
       </c>
+      <c r="AR266" t="n">
+        <v>267.2934265136719</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -37153,6 +37953,9 @@
       <c r="AQ267" t="n">
         <v>250.20458984375</v>
       </c>
+      <c r="AR267" t="n">
+        <v>253.4903411865234</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -37292,6 +38095,9 @@
       <c r="AQ268" t="n">
         <v>212.1442108154297</v>
       </c>
+      <c r="AR268" t="n">
+        <v>222.5008544921875</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -37429,6 +38235,9 @@
       <c r="AQ269" t="n">
         <v>201.7932434082031</v>
       </c>
+      <c r="AR269" t="n">
+        <v>202.5696563720703</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -37566,6 +38375,9 @@
       <c r="AQ270" t="n">
         <v>197.8139953613281</v>
       </c>
+      <c r="AR270" t="n">
+        <v>192.6471862792969</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -37703,6 +38515,9 @@
       <c r="AQ271" t="n">
         <v>193.4907836914062</v>
       </c>
+      <c r="AR271" t="n">
+        <v>185.4435272216797</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -37840,6 +38655,9 @@
       <c r="AQ272" t="n">
         <v>177.0764007568359</v>
       </c>
+      <c r="AR272" t="n">
+        <v>171.9967193603516</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -37977,6 +38795,9 @@
       <c r="AQ273" t="n">
         <v>166.4604034423828</v>
       </c>
+      <c r="AR273" t="n">
+        <v>162.6143798828125</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -38114,6 +38935,9 @@
       <c r="AQ274" t="n">
         <v>155.8182830810547</v>
       </c>
+      <c r="AR274" t="n">
+        <v>156.3444366455078</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -38251,6 +39075,9 @@
       <c r="AQ275" t="n">
         <v>135.1026306152344</v>
       </c>
+      <c r="AR275" t="n">
+        <v>132.5052795410156</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -38388,6 +39215,9 @@
       <c r="AQ276" t="n">
         <v>122.1054382324219</v>
       </c>
+      <c r="AR276" t="n">
+        <v>119.5272521972656</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="n">
@@ -38527,6 +39357,9 @@
       <c r="AQ277" t="n">
         <v>254.2998657226562</v>
       </c>
+      <c r="AR277" t="n">
+        <v>264.7604675292969</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="n">
@@ -38664,6 +39497,9 @@
       <c r="AQ278" t="n">
         <v>252.5075531005859</v>
       </c>
+      <c r="AR278" t="n">
+        <v>262.0411376953125</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="n">
@@ -38803,6 +39639,9 @@
       <c r="AQ279" t="n">
         <v>248.7033996582031</v>
       </c>
+      <c r="AR279" t="n">
+        <v>255.9441833496094</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="n">
@@ -38942,6 +39781,9 @@
       <c r="AQ280" t="n">
         <v>237.4970550537109</v>
       </c>
+      <c r="AR280" t="n">
+        <v>238.4380493164062</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="n">
@@ -39079,6 +39921,9 @@
       <c r="AQ281" t="n">
         <v>220.0389251708984</v>
       </c>
+      <c r="AR281" t="n">
+        <v>223.9438018798828</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="n">
@@ -39216,6 +40061,9 @@
       <c r="AQ282" t="n">
         <v>196.4653778076172</v>
       </c>
+      <c r="AR282" t="n">
+        <v>204.4272918701172</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="n">
@@ -39353,6 +40201,9 @@
       <c r="AQ283" t="n">
         <v>184.2713928222656</v>
       </c>
+      <c r="AR283" t="n">
+        <v>189.4378204345703</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="n">
@@ -39490,6 +40341,9 @@
       <c r="AQ284" t="n">
         <v>171.1510009765625</v>
       </c>
+      <c r="AR284" t="n">
+        <v>172.4234161376953</v>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="n">
@@ -39627,6 +40481,9 @@
       <c r="AQ285" t="n">
         <v>165.2402038574219</v>
       </c>
+      <c r="AR285" t="n">
+        <v>166.0079956054688</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="n">
@@ -39764,6 +40621,9 @@
       <c r="AQ286" t="n">
         <v>158.5668792724609</v>
       </c>
+      <c r="AR286" t="n">
+        <v>159.2900390625</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="n">
@@ -39901,6 +40761,9 @@
       <c r="AQ287" t="n">
         <v>145.6466827392578</v>
       </c>
+      <c r="AR287" t="n">
+        <v>145.9087219238281</v>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="n">
@@ -40038,6 +40901,9 @@
       <c r="AQ288" t="n">
         <v>140.517578125</v>
       </c>
+      <c r="AR288" t="n">
+        <v>142.8998413085938</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="n">
@@ -40175,6 +41041,9 @@
       <c r="AQ289" t="n">
         <v>138.8091888427734</v>
       </c>
+      <c r="AR289" t="n">
+        <v>141.4929656982422</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="n">
@@ -40314,6 +41183,9 @@
       <c r="AQ290" t="n">
         <v>279.4481811523438</v>
       </c>
+      <c r="AR290" t="n">
+        <v>277.5794982910156</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="n">
@@ -40451,6 +41323,9 @@
       <c r="AQ291" t="n">
         <v>275.8828735351562</v>
       </c>
+      <c r="AR291" t="n">
+        <v>271.9520568847656</v>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="n">
@@ -40590,6 +41465,9 @@
       <c r="AQ292" t="n">
         <v>267.248046875</v>
       </c>
+      <c r="AR292" t="n">
+        <v>260.5089416503906</v>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="n">
@@ -40729,6 +41607,9 @@
       <c r="AQ293" t="n">
         <v>242.6558532714844</v>
       </c>
+      <c r="AR293" t="n">
+        <v>226.6694793701172</v>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="n">
@@ -40866,6 +41747,9 @@
       <c r="AQ294" t="n">
         <v>222.27001953125</v>
       </c>
+      <c r="AR294" t="n">
+        <v>210.3001251220703</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="n">
@@ -41003,6 +41887,9 @@
       <c r="AQ295" t="n">
         <v>197.7889251708984</v>
       </c>
+      <c r="AR295" t="n">
+        <v>195.3731536865234</v>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="n">
@@ -41140,6 +42027,9 @@
       <c r="AQ296" t="n">
         <v>183.8530883789062</v>
       </c>
+      <c r="AR296" t="n">
+        <v>183.4754486083984</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="n">
@@ -41277,6 +42167,9 @@
       <c r="AQ297" t="n">
         <v>172.8410186767578</v>
       </c>
+      <c r="AR297" t="n">
+        <v>172.9342346191406</v>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="n">
@@ -41414,6 +42307,9 @@
       <c r="AQ298" t="n">
         <v>172.2611999511719</v>
       </c>
+      <c r="AR298" t="n">
+        <v>175.46142578125</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="n">
@@ -41551,6 +42447,9 @@
       <c r="AQ299" t="n">
         <v>174.7925415039062</v>
       </c>
+      <c r="AR299" t="n">
+        <v>178.8392333984375</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="n">
@@ -41688,6 +42587,9 @@
       <c r="AQ300" t="n">
         <v>167.5591583251953</v>
       </c>
+      <c r="AR300" t="n">
+        <v>173.8292999267578</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="n">
@@ -41825,6 +42727,9 @@
       <c r="AQ301" t="n">
         <v>146.9811096191406</v>
       </c>
+      <c r="AR301" t="n">
+        <v>150.8760375976562</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="n">
@@ -41962,6 +42867,9 @@
       <c r="AQ302" t="n">
         <v>136.6243896484375</v>
       </c>
+      <c r="AR302" t="n">
+        <v>133.2872314453125</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="n">
@@ -42099,6 +43007,9 @@
       <c r="AQ303" t="n">
         <v>122.741813659668</v>
       </c>
+      <c r="AR303" t="n">
+        <v>122.4256134033203</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="n">
@@ -42236,6 +43147,9 @@
       <c r="AQ304" t="n">
         <v>116.2026214599609</v>
       </c>
+      <c r="AR304" t="n">
+        <v>116.0171356201172</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="n">
@@ -42371,6 +43285,9 @@
       <c r="AQ305" t="n">
         <v>114.9154968261719</v>
       </c>
+      <c r="AR305" t="n">
+        <v>114.6743774414062</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="n">
@@ -42510,6 +43427,9 @@
       <c r="AQ306" t="n">
         <v>268.0990905761719</v>
       </c>
+      <c r="AR306" t="n">
+        <v>262.7090148925781</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="n">
@@ -42647,6 +43567,9 @@
       <c r="AQ307" t="n">
         <v>248.4622497558594</v>
       </c>
+      <c r="AR307" t="n">
+        <v>244.7051696777344</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="n">
@@ -42786,6 +43709,9 @@
       <c r="AQ308" t="n">
         <v>241.7124938964844</v>
       </c>
+      <c r="AR308" t="n">
+        <v>237.5629119873047</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="n">
@@ -42925,6 +43851,9 @@
       <c r="AQ309" t="n">
         <v>234.3346862792969</v>
       </c>
+      <c r="AR309" t="n">
+        <v>231.5282287597656</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="n">
@@ -43062,6 +43991,9 @@
       <c r="AQ310" t="n">
         <v>229.8614044189453</v>
       </c>
+      <c r="AR310" t="n">
+        <v>226.9401550292969</v>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="n">
@@ -43199,6 +44131,9 @@
       <c r="AQ311" t="n">
         <v>226.5618743896484</v>
       </c>
+      <c r="AR311" t="n">
+        <v>222.4472045898438</v>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="n">
@@ -43336,6 +44271,9 @@
       <c r="AQ312" t="n">
         <v>224.2044067382812</v>
       </c>
+      <c r="AR312" t="n">
+        <v>220.0367126464844</v>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="n">
@@ -43471,6 +44409,9 @@
       <c r="AQ313" t="n">
         <v>223.8068389892578</v>
       </c>
+      <c r="AR313" t="n">
+        <v>219.690673828125</v>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="n">
@@ -43610,6 +44551,9 @@
       <c r="AQ314" t="n">
         <v>304.1614074707031</v>
       </c>
+      <c r="AR314" t="n">
+        <v>297.4662475585938</v>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="n">
@@ -43749,6 +44693,9 @@
       <c r="AQ315" t="n">
         <v>286.1842651367188</v>
       </c>
+      <c r="AR315" t="n">
+        <v>281.975830078125</v>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="n">
@@ -43888,6 +44835,9 @@
       <c r="AQ316" t="n">
         <v>273.3499450683594</v>
       </c>
+      <c r="AR316" t="n">
+        <v>270.1025695800781</v>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="n">
@@ -44027,6 +44977,9 @@
       <c r="AQ317" t="n">
         <v>260.5735473632812</v>
       </c>
+      <c r="AR317" t="n">
+        <v>258.0227355957031</v>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="n">
@@ -44166,6 +45119,9 @@
       <c r="AQ318" t="n">
         <v>249.2293853759766</v>
       </c>
+      <c r="AR318" t="n">
+        <v>249.7472991943359</v>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="n">
@@ -44303,6 +45259,9 @@
       <c r="AQ319" t="n">
         <v>242.3335266113281</v>
       </c>
+      <c r="AR319" t="n">
+        <v>242.0873870849609</v>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="n">
@@ -44440,6 +45399,9 @@
       <c r="AQ320" t="n">
         <v>231.5265655517578</v>
       </c>
+      <c r="AR320" t="n">
+        <v>231.7945404052734</v>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="n">
@@ -44577,6 +45539,9 @@
       <c r="AQ321" t="n">
         <v>209.0898590087891</v>
       </c>
+      <c r="AR321" t="n">
+        <v>208.1519470214844</v>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="n">
@@ -44714,6 +45679,9 @@
       <c r="AQ322" t="n">
         <v>193.2579650878906</v>
       </c>
+      <c r="AR322" t="n">
+        <v>191.9669036865234</v>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="n">
@@ -44853,6 +45821,9 @@
       <c r="AQ323" t="n">
         <v>272.0978698730469</v>
       </c>
+      <c r="AR323" t="n">
+        <v>270.27783203125</v>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="n">
@@ -44992,6 +45963,9 @@
       <c r="AQ324" t="n">
         <v>262.4006042480469</v>
       </c>
+      <c r="AR324" t="n">
+        <v>257.6022033691406</v>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="n">
@@ -45131,6 +46105,9 @@
       <c r="AQ325" t="n">
         <v>239.3243865966797</v>
       </c>
+      <c r="AR325" t="n">
+        <v>239.1536712646484</v>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="n">
@@ -45270,6 +46247,9 @@
       <c r="AQ326" t="n">
         <v>221.6175079345703</v>
       </c>
+      <c r="AR326" t="n">
+        <v>226.1965026855469</v>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="n">
@@ -45409,6 +46389,9 @@
       <c r="AQ327" t="n">
         <v>208.0278015136719</v>
       </c>
+      <c r="AR327" t="n">
+        <v>212.9052124023438</v>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="n">
@@ -45546,6 +46529,9 @@
       <c r="AQ328" t="n">
         <v>191.7260437011719</v>
       </c>
+      <c r="AR328" t="n">
+        <v>194.3676910400391</v>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="n">
@@ -45683,6 +46669,9 @@
       <c r="AQ329" t="n">
         <v>178.966552734375</v>
       </c>
+      <c r="AR329" t="n">
+        <v>179.5796661376953</v>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="n">
@@ -45820,6 +46809,9 @@
       <c r="AQ330" t="n">
         <v>135.8283996582031</v>
       </c>
+      <c r="AR330" t="n">
+        <v>136.9672393798828</v>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="n">
@@ -45957,6 +46949,9 @@
       <c r="AQ331" t="n">
         <v>99.42548370361328</v>
       </c>
+      <c r="AR331" t="n">
+        <v>99.48162841796875</v>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="n">
@@ -46092,6 +47087,9 @@
       <c r="AQ332" t="n">
         <v>79.10947418212891</v>
       </c>
+      <c r="AR332" t="n">
+        <v>79.28661346435547</v>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="n">
@@ -46231,6 +47229,9 @@
       <c r="AQ333" t="n">
         <v>293.0044555664062</v>
       </c>
+      <c r="AR333" t="n">
+        <v>289.9403381347656</v>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="n">
@@ -46370,6 +47371,9 @@
       <c r="AQ334" t="n">
         <v>275.3695373535156</v>
       </c>
+      <c r="AR334" t="n">
+        <v>272.9808654785156</v>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="n">
@@ -46509,6 +47513,9 @@
       <c r="AQ335" t="n">
         <v>246.03564453125</v>
       </c>
+      <c r="AR335" t="n">
+        <v>244.4936828613281</v>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="n">
@@ -46648,6 +47655,9 @@
       <c r="AQ336" t="n">
         <v>208.5116882324219</v>
       </c>
+      <c r="AR336" t="n">
+        <v>209.5461273193359</v>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="n">
@@ -46787,6 +47797,9 @@
       <c r="AQ337" t="n">
         <v>193.1574859619141</v>
       </c>
+      <c r="AR337" t="n">
+        <v>189.9149017333984</v>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="n">
@@ -46924,6 +47937,9 @@
       <c r="AQ338" t="n">
         <v>183.8545074462891</v>
       </c>
+      <c r="AR338" t="n">
+        <v>181.3549041748047</v>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="n">
@@ -47061,6 +48077,9 @@
       <c r="AQ339" t="n">
         <v>176.3187103271484</v>
       </c>
+      <c r="AR339" t="n">
+        <v>175.2120056152344</v>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="n">
@@ -47198,6 +48217,9 @@
       <c r="AQ340" t="n">
         <v>165.2212219238281</v>
       </c>
+      <c r="AR340" t="n">
+        <v>165.5256958007812</v>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="n">
@@ -47335,6 +48357,9 @@
       <c r="AQ341" t="n">
         <v>158.2026824951172</v>
       </c>
+      <c r="AR341" t="n">
+        <v>159.2185821533203</v>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="n">
@@ -47472,6 +48497,9 @@
       <c r="AQ342" t="n">
         <v>152.4202270507812</v>
       </c>
+      <c r="AR342" t="n">
+        <v>153.3164215087891</v>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="n">
@@ -47607,6 +48635,9 @@
       <c r="AQ343" t="n">
         <v>149.18798828125</v>
       </c>
+      <c r="AR343" t="n">
+        <v>150.6905975341797</v>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="n">
@@ -47744,6 +48775,9 @@
       <c r="AQ344" t="n">
         <v>301.3240661621094</v>
       </c>
+      <c r="AR344" t="n">
+        <v>303.7353515625</v>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="n">
@@ -47881,6 +48915,9 @@
       <c r="AQ345" t="n">
         <v>351.9208374023438</v>
       </c>
+      <c r="AR345" t="n">
+        <v>356.4658508300781</v>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="n">
@@ -48020,6 +49057,9 @@
       <c r="AQ346" t="n">
         <v>248.7835998535156</v>
       </c>
+      <c r="AR346" t="n">
+        <v>239.0724487304688</v>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="n">
@@ -48159,6 +49199,9 @@
       <c r="AQ347" t="n">
         <v>110.5615692138672</v>
       </c>
+      <c r="AR347" t="n">
+        <v>110.2445755004883</v>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="n">
@@ -48298,6 +49341,9 @@
       <c r="AQ348" t="n">
         <v>304.3471374511719</v>
       </c>
+      <c r="AR348" t="n">
+        <v>304.6908569335938</v>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="n">
@@ -48437,6 +49483,9 @@
       <c r="AQ349" t="n">
         <v>349.4158935546875</v>
       </c>
+      <c r="AR349" t="n">
+        <v>351.7840881347656</v>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="n">
@@ -48576,6 +49625,9 @@
       <c r="AQ350" t="n">
         <v>385.1006469726562</v>
       </c>
+      <c r="AR350" t="n">
+        <v>386.0926513671875</v>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="n">
@@ -48715,6 +49767,9 @@
       <c r="AQ351" t="n">
         <v>245.3583679199219</v>
       </c>
+      <c r="AR351" t="n">
+        <v>247.9981994628906</v>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="n">
@@ -48854,6 +49909,9 @@
       <c r="AQ352" t="n">
         <v>201.5950622558594</v>
       </c>
+      <c r="AR352" t="n">
+        <v>192.7016143798828</v>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="n">
@@ -48991,6 +50049,9 @@
       <c r="AQ353" t="n">
         <v>191.7413330078125</v>
       </c>
+      <c r="AR353" t="n">
+        <v>184.3531799316406</v>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="n">
@@ -49128,6 +50189,9 @@
       <c r="AQ354" t="n">
         <v>180.9402923583984</v>
       </c>
+      <c r="AR354" t="n">
+        <v>180.3672790527344</v>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="n">
@@ -49265,6 +50329,9 @@
       <c r="AQ355" t="n">
         <v>169.1606140136719</v>
       </c>
+      <c r="AR355" t="n">
+        <v>168.1485748291016</v>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="n">
@@ -49402,6 +50469,9 @@
       <c r="AQ356" t="n">
         <v>157.1785736083984</v>
       </c>
+      <c r="AR356" t="n">
+        <v>159.5711517333984</v>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="n">
@@ -49539,6 +50609,9 @@
       <c r="AQ357" t="n">
         <v>142.9977416992188</v>
       </c>
+      <c r="AR357" t="n">
+        <v>140.9219818115234</v>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="n">
@@ -49676,6 +50749,9 @@
       <c r="AQ358" t="n">
         <v>100.3862991333008</v>
       </c>
+      <c r="AR358" t="n">
+        <v>100.5576629638672</v>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="n">
@@ -49815,6 +50891,9 @@
       <c r="AQ359" t="n">
         <v>303.5867309570312</v>
       </c>
+      <c r="AR359" t="n">
+        <v>312.5636596679688</v>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="n">
@@ -49954,6 +51033,9 @@
       <c r="AQ360" t="n">
         <v>363.8936462402344</v>
       </c>
+      <c r="AR360" t="n">
+        <v>364.1470336914062</v>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="n">
@@ -50093,6 +51175,9 @@
       <c r="AQ361" t="n">
         <v>367.1419677734375</v>
       </c>
+      <c r="AR361" t="n">
+        <v>369.4036865234375</v>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="n">
@@ -50232,6 +51317,9 @@
       <c r="AQ362" t="n">
         <v>243.2415771484375</v>
       </c>
+      <c r="AR362" t="n">
+        <v>255.5150299072266</v>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="n">
@@ -50371,6 +51459,9 @@
       <c r="AQ363" t="n">
         <v>211.2501831054688</v>
       </c>
+      <c r="AR363" t="n">
+        <v>210.293212890625</v>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="n">
@@ -50508,6 +51599,9 @@
       <c r="AQ364" t="n">
         <v>204.0858612060547</v>
       </c>
+      <c r="AR364" t="n">
+        <v>204.3328094482422</v>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="n">
@@ -50645,6 +51739,9 @@
       <c r="AQ365" t="n">
         <v>200.0545806884766</v>
       </c>
+      <c r="AR365" t="n">
+        <v>200.0346832275391</v>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="n">
@@ -50782,6 +51879,9 @@
       <c r="AQ366" t="n">
         <v>196.220458984375</v>
       </c>
+      <c r="AR366" t="n">
+        <v>195.1361083984375</v>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="n">
@@ -50919,6 +52019,9 @@
       <c r="AQ367" t="n">
         <v>194.7718811035156</v>
       </c>
+      <c r="AR367" t="n">
+        <v>192.1937255859375</v>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="n">
@@ -51056,6 +52159,9 @@
       <c r="AQ368" t="n">
         <v>158.6254577636719</v>
       </c>
+      <c r="AR368" t="n">
+        <v>158.3020782470703</v>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="n">
@@ -51192,6 +52298,9 @@
       </c>
       <c r="AQ369" t="n">
         <v>106.0043716430664</v>
+      </c>
+      <c r="AR369" t="n">
+        <v>105.0265808105469</v>
       </c>
     </row>
   </sheetData>

</xml_diff>